<commit_message>
Đổi tên tư vấn giám sát Trần Mạnh Tùng thành Lê Quốc Huy trong hồ sơ XD8 và XD4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RHahmApFFRr7mqf4R5YZ3w
</commit_message>
<xml_diff>
--- a/XD4/Đoạn 1/1. Danh mục nghiệm thu - XD4 đoạn 1.xlsx
+++ b/XD4/Đoạn 1/1. Danh mục nghiệm thu - XD4 đoạn 1.xlsx
@@ -161,7 +161,7 @@
     <t xml:space="preserve">Nguyễn Xuân Hưng</t>
   </si>
   <si>
-    <t xml:space="preserve">Trần Mạnh Tùng</t>
+    <t xml:space="preserve">Lê Quốc Huy</t>
   </si>
   <si>
     <t xml:space="preserve">Đào đất xử lý nền đường đoạn từ Km0+441,84 - Km0+554,08</t>
@@ -15886,7 +15886,7 @@
       <c r="J57" s="71"/>
       <c r="K57" s="71" t="str">
         <f aca="false">'Tuyến XD4'!Q3</f>
-        <v>Trần Mạnh Tùng</v>
+        <v>Lê Quốc Huy</v>
       </c>
       <c r="L57" s="71"/>
       <c r="M57" s="71"/>
@@ -18027,7 +18027,7 @@
       <c r="N68" s="87"/>
       <c r="O68" s="71" t="str">
         <f aca="false">'1. PL đường đen'!K57</f>
-        <v>Trần Mạnh Tùng</v>
+        <v>Lê Quốc Huy</v>
       </c>
       <c r="P68" s="71"/>
       <c r="Q68" s="71"/>
@@ -20280,7 +20280,7 @@
       <c r="D58" s="122"/>
       <c r="E58" s="71" t="str">
         <f aca="false">+'2. Cao độ đào nền'!O68</f>
-        <v>Trần Mạnh Tùng</v>
+        <v>Lê Quốc Huy</v>
       </c>
       <c r="F58" s="71"/>
       <c r="G58" s="71"/>

</xml_diff>